<commit_message>
Changing paths based on new logic
</commit_message>
<xml_diff>
--- a/data/clean_data/declaraciones/compiled_dataset_filtered.xlsx
+++ b/data/clean_data/declaraciones/compiled_dataset_filtered.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,107 +433,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>fecha_creación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>fecha_modificacion</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ejercicio</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>fecha_informa</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>fecha_termino_informe</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tipo_integrante</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>nivel_puesto</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>puesto_perspectiva_genero</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>denominacion</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>area</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>primer_apellido</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>segundo_apellido</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>sexo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>modalidad</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>hipervinculo</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>responsable</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>fecha_actualizacion</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>nota</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
@@ -531,19 +543,19 @@
       <c r="A2" t="n">
         <v>2207615525</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>45413</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>45624</v>
       </c>
       <c r="D2" t="n">
         <v>2024</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>45292</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>45382</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -602,7 +614,7 @@
           <t>DirecciÔøΩn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S2" s="1" t="n">
+      <c r="S2" s="2" t="n">
         <v>45334</v>
       </c>
       <c r="T2" t="inlineStr">
@@ -620,19 +632,19 @@
       <c r="A3" t="n">
         <v>2207615528</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>45413</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>45624</v>
       </c>
       <c r="D3" t="n">
         <v>2024</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>45292</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>45382</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -691,7 +703,7 @@
           <t>DirecciÔøΩn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S3" s="1" t="n">
+      <c r="S3" s="2" t="n">
         <v>45305</v>
       </c>
       <c r="T3" t="inlineStr">
@@ -709,19 +721,19 @@
       <c r="A4" t="n">
         <v>2422696423</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="D4" t="n">
         <v>2025</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>45658</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -780,7 +792,7 @@
           <t>DirecciÔøΩn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S4" s="1" t="n">
+      <c r="S4" s="2" t="n">
         <v>45667</v>
       </c>
       <c r="T4" t="inlineStr">
@@ -798,19 +810,19 @@
       <c r="A5" t="n">
         <v>2301653179</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D5" t="n">
         <v>2024</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -869,7 +881,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S5" s="1" t="n">
+      <c r="S5" s="2" t="n">
         <v>45441</v>
       </c>
       <c r="T5" t="inlineStr">
@@ -887,19 +899,19 @@
       <c r="A6" t="n">
         <v>2301653189</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D6" t="n">
         <v>2024</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -958,7 +970,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S6" s="1" t="n">
+      <c r="S6" s="2" t="n">
         <v>45443</v>
       </c>
       <c r="T6" t="inlineStr">
@@ -976,19 +988,19 @@
       <c r="A7" t="n">
         <v>2301653185</v>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D7" t="n">
         <v>2024</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -1047,7 +1059,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S7" s="1" t="n">
+      <c r="S7" s="2" t="n">
         <v>45433</v>
       </c>
       <c r="T7" t="inlineStr">
@@ -1065,19 +1077,19 @@
       <c r="A8" t="n">
         <v>2301653187</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D8" t="n">
         <v>2024</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -1136,7 +1148,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S8" s="1" t="n">
+      <c r="S8" s="2" t="n">
         <v>45441</v>
       </c>
       <c r="T8" t="inlineStr">
@@ -1154,19 +1166,19 @@
       <c r="A9" t="n">
         <v>2301653188</v>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D9" t="n">
         <v>2024</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -1225,7 +1237,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S9" s="1" t="n">
+      <c r="S9" s="2" t="n">
         <v>45436</v>
       </c>
       <c r="T9" t="inlineStr">
@@ -1243,19 +1255,19 @@
       <c r="A10" t="n">
         <v>2301653180</v>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D10" t="n">
         <v>2024</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -1314,7 +1326,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S10" s="1" t="n">
+      <c r="S10" s="2" t="n">
         <v>45439</v>
       </c>
       <c r="T10" t="inlineStr">
@@ -1332,19 +1344,19 @@
       <c r="A11" t="n">
         <v>2301653182</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D11" t="n">
         <v>2024</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -1403,7 +1415,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S11" s="1" t="n">
+      <c r="S11" s="2" t="n">
         <v>45442</v>
       </c>
       <c r="T11" t="inlineStr">
@@ -1421,19 +1433,19 @@
       <c r="A12" t="n">
         <v>2301653184</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D12" t="n">
         <v>2024</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -1492,7 +1504,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S12" s="1" t="n">
+      <c r="S12" s="2" t="n">
         <v>45439</v>
       </c>
       <c r="T12" t="inlineStr">
@@ -1510,19 +1522,19 @@
       <c r="A13" t="n">
         <v>2301653181</v>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D13" t="n">
         <v>2024</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1581,7 +1593,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S13" s="1" t="n">
+      <c r="S13" s="2" t="n">
         <v>45440</v>
       </c>
       <c r="T13" t="inlineStr">
@@ -1599,19 +1611,19 @@
       <c r="A14" t="n">
         <v>2301653186</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D14" t="n">
         <v>2024</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -1670,7 +1682,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S14" s="1" t="n">
+      <c r="S14" s="2" t="n">
         <v>45437</v>
       </c>
       <c r="T14" t="inlineStr">
@@ -1688,19 +1700,19 @@
       <c r="A15" t="n">
         <v>2301653183</v>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="2" t="n">
         <v>45488</v>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>45618</v>
       </c>
       <c r="D15" t="n">
         <v>2024</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1759,7 +1771,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S15" s="1" t="n">
+      <c r="S15" s="2" t="n">
         <v>45434</v>
       </c>
       <c r="T15" t="inlineStr">
@@ -1777,19 +1789,19 @@
       <c r="A16" t="n">
         <v>2439396595</v>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D16" t="n">
         <v>2025</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1848,7 +1860,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S16" s="1" t="n">
+      <c r="S16" s="2" t="n">
         <v>45797</v>
       </c>
       <c r="T16" t="inlineStr">
@@ -1866,19 +1878,19 @@
       <c r="A17" t="n">
         <v>2439396589</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D17" t="n">
         <v>2025</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1937,7 +1949,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S17" s="1" t="n">
+      <c r="S17" s="2" t="n">
         <v>45807</v>
       </c>
       <c r="T17" t="inlineStr">
@@ -1955,19 +1967,19 @@
       <c r="A18" t="n">
         <v>2439396593</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D18" t="n">
         <v>2025</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G18" t="inlineStr">
@@ -2026,7 +2038,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S18" s="1" t="n">
+      <c r="S18" s="2" t="n">
         <v>45806</v>
       </c>
       <c r="T18" t="inlineStr">
@@ -2044,19 +2056,19 @@
       <c r="A19" t="n">
         <v>2439396586</v>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D19" t="n">
         <v>2025</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G19" t="inlineStr">
@@ -2115,7 +2127,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S19" s="1" t="n">
+      <c r="S19" s="2" t="n">
         <v>45806</v>
       </c>
       <c r="T19" t="inlineStr">
@@ -2133,19 +2145,19 @@
       <c r="A20" t="n">
         <v>2439396594</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D20" t="n">
         <v>2025</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G20" t="inlineStr">
@@ -2204,7 +2216,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S20" s="1" t="n">
+      <c r="S20" s="2" t="n">
         <v>45808</v>
       </c>
       <c r="T20" t="inlineStr">
@@ -2222,19 +2234,19 @@
       <c r="A21" t="n">
         <v>2439396588</v>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D21" t="n">
         <v>2025</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="F21" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -2293,7 +2305,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S21" s="1" t="n">
+      <c r="S21" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="T21" t="inlineStr">
@@ -2311,19 +2323,19 @@
       <c r="A22" t="n">
         <v>2439396591</v>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D22" t="n">
         <v>2025</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -2382,7 +2394,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S22" s="1" t="n">
+      <c r="S22" s="2" t="n">
         <v>45805</v>
       </c>
       <c r="T22" t="inlineStr">
@@ -2400,19 +2412,19 @@
       <c r="A23" t="n">
         <v>2439396587</v>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D23" t="n">
         <v>2025</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -2471,7 +2483,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S23" s="1" t="n">
+      <c r="S23" s="2" t="n">
         <v>45800</v>
       </c>
       <c r="T23" t="inlineStr">
@@ -2489,19 +2501,19 @@
       <c r="A24" t="n">
         <v>2439396590</v>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D24" t="n">
         <v>2025</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G24" t="inlineStr">
@@ -2560,7 +2572,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S24" s="1" t="n">
+      <c r="S24" s="2" t="n">
         <v>45803</v>
       </c>
       <c r="T24" t="inlineStr">
@@ -2578,19 +2590,19 @@
       <c r="A25" t="n">
         <v>2439396592</v>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" s="2" t="n">
         <v>45854</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>45854</v>
       </c>
       <c r="D25" t="n">
         <v>2025</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="G25" t="inlineStr">
@@ -2649,7 +2661,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S25" s="1" t="n">
+      <c r="S25" s="2" t="n">
         <v>45806</v>
       </c>
       <c r="T25" t="inlineStr">
@@ -2667,19 +2679,19 @@
       <c r="A26" t="n">
         <v>2516992219</v>
       </c>
-      <c r="B26" s="1" t="n">
+      <c r="B26" s="2" t="n">
         <v>45961</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="D26" t="n">
         <v>2025</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -2738,7 +2750,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S26" s="1" t="n">
+      <c r="S26" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="T26" t="inlineStr">
@@ -2756,19 +2768,19 @@
       <c r="A27" t="n">
         <v>2516992222</v>
       </c>
-      <c r="B27" s="1" t="n">
+      <c r="B27" s="2" t="n">
         <v>45961</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="D27" t="n">
         <v>2025</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="G27" t="inlineStr">
@@ -2827,7 +2839,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S27" s="1" t="n">
+      <c r="S27" s="2" t="n">
         <v>45923</v>
       </c>
       <c r="T27" t="inlineStr">
@@ -2845,19 +2857,19 @@
       <c r="A28" t="n">
         <v>2516992221</v>
       </c>
-      <c r="B28" s="1" t="n">
+      <c r="B28" s="2" t="n">
         <v>45961</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="D28" t="n">
         <v>2025</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -2916,7 +2928,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S28" s="1" t="n">
+      <c r="S28" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="T28" t="inlineStr">
@@ -2934,19 +2946,19 @@
       <c r="A29" t="n">
         <v>2516992218</v>
       </c>
-      <c r="B29" s="1" t="n">
+      <c r="B29" s="2" t="n">
         <v>45961</v>
       </c>
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="D29" t="n">
         <v>2025</v>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="F29" s="1" t="n">
+      <c r="F29" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="G29" t="inlineStr">
@@ -3005,7 +3017,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S29" s="1" t="n">
+      <c r="S29" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="T29" t="inlineStr">
@@ -3023,19 +3035,19 @@
       <c r="A30" t="n">
         <v>2516992220</v>
       </c>
-      <c r="B30" s="1" t="n">
+      <c r="B30" s="2" t="n">
         <v>45961</v>
       </c>
-      <c r="C30" s="1" t="n">
+      <c r="C30" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="D30" t="n">
         <v>2025</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="F30" s="1" t="n">
+      <c r="F30" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="G30" t="inlineStr">
@@ -3094,7 +3106,7 @@
           <t>DirecciÛn General de Responsabilidades Administrativas y de Registro Patrimonial</t>
         </is>
       </c>
-      <c r="S30" s="1" t="n">
+      <c r="S30" s="2" t="n">
         <v>45898</v>
       </c>
       <c r="T30" t="inlineStr">

</xml_diff>